<commit_message>
Update: Penambahan dan Normalisasi 'Kode Unit Kerja' sebagai salah satu key parameter
</commit_message>
<xml_diff>
--- a/exports/formatTabelS14.xlsx
+++ b/exports/formatTabelS14.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MonitoringHukdis_Zip\exports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C05693-05FB-4D35-8EF4-0FD95EF02501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27EB1376-AEDE-4581-8887-FAD416F42B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3DAB9FA1-7F3C-445D-B3BD-4FB35A43BC4B}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6817" uniqueCount="684">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6841" uniqueCount="685">
   <si>
     <t>no</t>
   </si>
@@ -2075,6 +2075,9 @@
   </si>
   <si>
     <t>pertimbangan_rekomendasi_uka_dengan_s14</t>
+  </si>
+  <si>
+    <t>KC BSD</t>
   </si>
 </sst>
 </file>
@@ -2920,7 +2923,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7391526F-3277-4980-A0D5-696D0CDBD6DB}">
-  <dimension ref="A1:AJ300"/>
+  <dimension ref="A1:AJ301"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="18" max="18" width="28.7265625" bestFit="1" customWidth="1"/>
@@ -31074,6 +31077,104 @@
         <v>52</v>
       </c>
     </row>
+    <row r="301" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A301">
+        <v>4</v>
+      </c>
+      <c r="B301" t="s">
+        <v>213</v>
+      </c>
+      <c r="C301">
+        <v>2024</v>
+      </c>
+      <c r="D301" t="s">
+        <v>36</v>
+      </c>
+      <c r="E301" t="s">
+        <v>666</v>
+      </c>
+      <c r="F301" s="1">
+        <v>45423</v>
+      </c>
+      <c r="G301" t="s">
+        <v>647</v>
+      </c>
+      <c r="H301">
+        <v>1638955408</v>
+      </c>
+      <c r="I301">
+        <v>504</v>
+      </c>
+      <c r="J301" t="s">
+        <v>684</v>
+      </c>
+      <c r="K301">
+        <v>95595</v>
+      </c>
+      <c r="L301" t="s">
+        <v>681</v>
+      </c>
+      <c r="M301" t="s">
+        <v>182</v>
+      </c>
+      <c r="N301" t="s">
+        <v>182</v>
+      </c>
+      <c r="O301">
+        <v>7</v>
+      </c>
+      <c r="P301" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q301" t="s">
+        <v>59</v>
+      </c>
+      <c r="R301" t="s">
+        <v>43</v>
+      </c>
+      <c r="S301" s="2">
+        <v>45302</v>
+      </c>
+      <c r="T301" t="s">
+        <v>45</v>
+      </c>
+      <c r="U301" t="s">
+        <v>44</v>
+      </c>
+      <c r="V301" t="s">
+        <v>45</v>
+      </c>
+      <c r="W301" t="s">
+        <v>45</v>
+      </c>
+      <c r="X301" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y301" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z301" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA301" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB301" t="s">
+        <v>682</v>
+      </c>
+      <c r="AC301" t="s">
+        <v>50</v>
+      </c>
+      <c r="AD301" t="s">
+        <v>84</v>
+      </c>
+      <c r="AE301" t="s">
+        <v>51</v>
+      </c>
+      <c r="AF301" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AJ300" xr:uid="{7391526F-3277-4980-A0D5-696D0CDBD6DB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>